<commit_message>
refactor: remove base parameter from set_Model, drop .CR_Base
set_Model() no longer needs base — JSON config handles everything for
both built-in and custom models. RR_std() now uses .CR_Model directly.
Removed IER prefix fallback since all variants have their own JSON entries.
</commit_message>
<xml_diff>
--- a/Data/RR_index/NO2_CR_Lookup_Table.xlsx
+++ b/Data/RR_index/NO2_CR_Lookup_Table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20338"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mygit\O3-attr-mort\Data\RR_index\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitDir\PM2.5-attr-mort\Data\RR_index\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{884269B1-DDBC-42DF-8930-CB531236B2CC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51575DB3-4C15-4955-9955-9495D00719BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LOW" sheetId="1" r:id="rId1"/>
@@ -18,16 +18,25 @@
     <sheet name="UP" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="179021"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
   <si>
     <t>concentration</t>
   </si>
   <si>
     <t>CAUSE_ALL</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ALLCAUSE_ALL</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -119,9 +128,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -159,9 +168,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -194,26 +203,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -246,26 +238,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -450,7 +425,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
feat: set_Model(path=...) auto-appends config entry to RR_std_config.json
Reads existing JSON, inserts new model entry before the closing brace.
Skips if model already exists. Creates the file if absent.
</commit_message>
<xml_diff>
--- a/Data/RR_index/NO2_CR_Lookup_Table.xlsx
+++ b/Data/RR_index/NO2_CR_Lookup_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitDir\PM2.5-attr-mort\Data\RR_index\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51575DB3-4C15-4955-9955-9495D00719BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE79A65-1F8D-4CA2-AD01-FA06262D83B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LOW" sheetId="1" r:id="rId1"/>
@@ -27,13 +27,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="2">
   <si>
     <t>concentration</t>
-  </si>
-  <si>
-    <t>CAUSE_ALL</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>ALLCAUSE_ALL</t>
@@ -425,7 +421,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.15">

</xml_diff>